<commit_message>
Add Excel Scenario Lab — compare full plans side by side
Mirror the web app's Compare tab in the workbook: rebuild the Scenarios
sheet into a side-by-side Scenario Lab.

- Six scenario columns (Base/Bull/Bear + three open slots), each with its
  own editable dials: price/can, cost/can, cases/year, trade level, marketing.
- Live formula rows per column (net sales, gross margin %, contribution %,
  break-even cases, EBITDA $ and %), derived from the channel totals via
  hidden multiplier helper rows.
- Best number in each row highlighted green (FormulaRule MAX/MIN); EBITDA
  red/green font; EBITDA-by-scenario bar chart.

Verified with the `formulas` engine: the Base column reconciles to the
dollar with the web app and the rest of the workbook (net $4,961,478,
EBITDA -$648,238, break-even 415,070); Bull +$382K, Bear -$1.18M; existing
sheets unaffected.

https://claude.ai/code/session_01XtU4ZhhiP3B25DcbgYH1Pu
</commit_message>
<xml_diff>
--- a/organika-cpg-pnl.xlsx
+++ b/organika-cpg-pnl.xlsx
@@ -11,7 +11,7 @@
     <sheet name="COGS_BOM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Channels" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Scenario Lab" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Guide" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
@@ -27,7 +27,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -150,6 +150,18 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00222222"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0093A0BA"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="002BB3A3"/>
       <sz val="12"/>
     </font>
@@ -222,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -354,36 +366,45 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -397,6 +418,27 @@
           <fgColor rgb="0063BE7B"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E4F7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00C00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="001F9E6E"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -471,6 +513,80 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>EBITDA by scenario</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Scenario Lab'!$C$11:$H$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Scenario Lab'!$C$22:$H$22</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -524,6 +640,33 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2672,325 +2815,593 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Scenario planning — Base / Bull / Bear</t>
+          <t>Scenario Lab — compare full plans side by side</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bull and Bear scale your Base assumptions. Multipliers are editable; metrics derive from the channel totals.</t>
+          <t>Each column is a plan. Edit the yellow dials; results recompute live and the best in each row turns green.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="45" t="inlineStr">
-        <is>
-          <t>Multiplier</t>
-        </is>
-      </c>
-      <c r="C4" s="46" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="D4" s="46" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="E4" s="46" t="inlineStr">
-        <is>
-          <t>Bear</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>MODEL BASIS (LIVE, FROM YOUR PLAN)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Volume ×</t>
-        </is>
-      </c>
-      <c r="C5" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="47" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E5" s="47" t="n">
-        <v>0.75</v>
+          <t>Base price / can</t>
+        </is>
+      </c>
+      <c r="C5" s="45">
+        <f>Channels!$L$9/Channels!$K$9</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Price ×</t>
-        </is>
-      </c>
-      <c r="C6" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="47" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="E6" s="47" t="n">
-        <v>0.97</v>
+          <t>Base cost / can</t>
+        </is>
+      </c>
+      <c r="C6" s="24">
+        <f>COGS_BOM!$C$41</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>COGS ×</t>
-        </is>
-      </c>
-      <c r="C7" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="47" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E7" s="47" t="n">
-        <v>1.1</v>
+          <t>Base volume (cases)</t>
+        </is>
+      </c>
+      <c r="C7" s="6">
+        <f>'P&amp;L'!$C$5</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Trade ×</t>
-        </is>
-      </c>
-      <c r="C8" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="47" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="E8" s="47" t="n">
-        <v>1.15</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Ad / CAC ×</t>
-        </is>
-      </c>
-      <c r="C9" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="47" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="E9" s="47" t="n">
-        <v>1.2</v>
+          <t>Fixed costs</t>
+        </is>
+      </c>
+      <c r="C8" s="46">
+        <f>'P&amp;L'!$C$13</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>RESULTING P&amp;L</t>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="F11" s="47" t="inlineStr">
+        <is>
+          <t>Scenario 4</t>
+        </is>
+      </c>
+      <c r="G11" s="47" t="inlineStr">
+        <is>
+          <t>Scenario 5</t>
+        </is>
+      </c>
+      <c r="H11" s="47" t="inlineStr">
+        <is>
+          <t>Scenario 6</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>Bear</t>
-        </is>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Price / can</t>
+        </is>
+      </c>
+      <c r="C12" s="48" t="n">
+        <v>1.919</v>
+      </c>
+      <c r="D12" s="48" t="n">
+        <v>2.015</v>
+      </c>
+      <c r="E12" s="48" t="n">
+        <v>1.861</v>
+      </c>
+      <c r="F12" s="48" t="n">
+        <v>1.919</v>
+      </c>
+      <c r="G12" s="48" t="n">
+        <v>1.919</v>
+      </c>
+      <c r="H12" s="48" t="n">
+        <v>1.919</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Annual cases</t>
-        </is>
-      </c>
-      <c r="C13" s="48">
-        <f>'P&amp;L'!$C$5*C5</f>
-        <v/>
-      </c>
-      <c r="D13" s="48">
-        <f>'P&amp;L'!$C$5*D5</f>
-        <v/>
-      </c>
-      <c r="E13" s="48">
-        <f>'P&amp;L'!$C$5*E5</f>
-        <v/>
+          <t>Cost / can</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>0.58125</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>0.52313</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>0.6393799999999999</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.58125</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>0.58125</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>0.58125</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Net sales</t>
-        </is>
-      </c>
-      <c r="C14" s="14">
-        <f>(C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="D14" s="14">
-        <f>(D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="E14" s="14">
-        <f>(E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
+          <t>Cases / year</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>350000</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>187500</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>250000</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>250000</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Gross margin %</t>
-        </is>
-      </c>
-      <c r="C15" s="49">
-        <f>((C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-C7*C5*Channels!$P$9)/(C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="D15" s="49">
-        <f>((D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-D7*D5*Channels!$P$9)/(D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="E15" s="49">
-        <f>((E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-E7*E5*Channels!$P$9)/(E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
+          <t>Trade level (×)</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E15" s="49" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="F15" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Contribution $</t>
-        </is>
-      </c>
-      <c r="C16" s="14">
-        <f>(((C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-C7*C5*Channels!$P$9)-C6*C5*Channels!$R$9-C9*C6*C5*Channels!$S$9-C5*Channels!$T$9-C5*Channels!$U$9)</f>
-        <v/>
-      </c>
-      <c r="D16" s="14">
-        <f>(((D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-D7*D5*Channels!$P$9)-D6*D5*Channels!$R$9-D9*D6*D5*Channels!$S$9-D5*Channels!$T$9-D5*Channels!$U$9)</f>
-        <v/>
-      </c>
-      <c r="E16" s="14">
-        <f>(((E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-E7*E5*Channels!$P$9)-E6*E5*Channels!$R$9-E9*E6*E5*Channels!$S$9-E5*Channels!$T$9-E5*Channels!$U$9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="4" t="inlineStr">
+          <t>Marketing (% net)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Net sales</t>
+        </is>
+      </c>
+      <c r="C18" s="14">
+        <f>C25*C27*(Channels!$L$9-C15*Channels!$M$9-Channels!$N$9)</f>
+        <v/>
+      </c>
+      <c r="D18" s="14">
+        <f>D25*D27*(Channels!$L$9-D15*Channels!$M$9-Channels!$N$9)</f>
+        <v/>
+      </c>
+      <c r="E18" s="14">
+        <f>E25*E27*(Channels!$L$9-E15*Channels!$M$9-Channels!$N$9)</f>
+        <v/>
+      </c>
+      <c r="F18" s="14">
+        <f>F25*F27*(Channels!$L$9-F15*Channels!$M$9-Channels!$N$9)</f>
+        <v/>
+      </c>
+      <c r="G18" s="14">
+        <f>G25*G27*(Channels!$L$9-G15*Channels!$M$9-Channels!$N$9)</f>
+        <v/>
+      </c>
+      <c r="H18" s="14">
+        <f>H25*H27*(Channels!$L$9-H15*Channels!$M$9-Channels!$N$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="C19" s="50">
+        <f>(C18-C26*C27*Channels!$P$9)/C18</f>
+        <v/>
+      </c>
+      <c r="D19" s="50">
+        <f>(D18-D26*D27*Channels!$P$9)/D18</f>
+        <v/>
+      </c>
+      <c r="E19" s="50">
+        <f>(E18-E26*E27*Channels!$P$9)/E18</f>
+        <v/>
+      </c>
+      <c r="F19" s="50">
+        <f>(F18-F26*F27*Channels!$P$9)/F18</f>
+        <v/>
+      </c>
+      <c r="G19" s="50">
+        <f>(G18-G26*G27*Channels!$P$9)/G18</f>
+        <v/>
+      </c>
+      <c r="H19" s="50">
+        <f>(H18-H26*H27*Channels!$P$9)/H18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Contribution %</t>
         </is>
       </c>
-      <c r="C17" s="49">
-        <f>(((C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-C7*C5*Channels!$P$9)-C6*C5*Channels!$R$9-C9*C6*C5*Channels!$S$9-C5*Channels!$T$9-C5*Channels!$U$9)/(C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="D17" s="49">
-        <f>(((D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-D7*D5*Channels!$P$9)-D6*D5*Channels!$R$9-D9*D6*D5*Channels!$S$9-D5*Channels!$T$9-D5*Channels!$U$9)/(D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="E17" s="49">
-        <f>(((E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-E7*E5*Channels!$P$9)-E6*E5*Channels!$R$9-E9*E6*E5*Channels!$S$9-E5*Channels!$T$9-E5*Channels!$U$9)/(E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>EBITDA $</t>
-        </is>
-      </c>
-      <c r="C18" s="50">
-        <f>((((C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-C7*C5*Channels!$P$9)-C6*C5*Channels!$R$9-C9*C6*C5*Channels!$S$9-C5*Channels!$T$9-C5*Channels!$U$9)-'P&amp;L'!$C$8*(C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-'P&amp;L'!$C$13)</f>
-        <v/>
-      </c>
-      <c r="D18" s="50">
-        <f>((((D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-D7*D5*Channels!$P$9)-D6*D5*Channels!$R$9-D9*D6*D5*Channels!$S$9-D5*Channels!$T$9-D5*Channels!$U$9)-'P&amp;L'!$C$8*(D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-'P&amp;L'!$C$13)</f>
-        <v/>
-      </c>
-      <c r="E18" s="50">
-        <f>((((E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-E7*E5*Channels!$P$9)-E6*E5*Channels!$R$9-E9*E6*E5*Channels!$S$9-E5*Channels!$T$9-E5*Channels!$U$9)-'P&amp;L'!$C$8*(E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-'P&amp;L'!$C$13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="9" t="inlineStr">
+      <c r="C20" s="50">
+        <f>C28/C18</f>
+        <v/>
+      </c>
+      <c r="D20" s="50">
+        <f>D28/D18</f>
+        <v/>
+      </c>
+      <c r="E20" s="50">
+        <f>E28/E18</f>
+        <v/>
+      </c>
+      <c r="F20" s="50">
+        <f>F28/F18</f>
+        <v/>
+      </c>
+      <c r="G20" s="50">
+        <f>G28/G18</f>
+        <v/>
+      </c>
+      <c r="H20" s="50">
+        <f>H28/H18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Break-even (cases)</t>
+        </is>
+      </c>
+      <c r="C21" s="51">
+        <f>IF((C22+$C$8)&gt;0,$C$8*C14/(C22+$C$8),"n/a")</f>
+        <v/>
+      </c>
+      <c r="D21" s="51">
+        <f>IF((D22+$C$8)&gt;0,$C$8*D14/(D22+$C$8),"n/a")</f>
+        <v/>
+      </c>
+      <c r="E21" s="51">
+        <f>IF((E22+$C$8)&gt;0,$C$8*E14/(E22+$C$8),"n/a")</f>
+        <v/>
+      </c>
+      <c r="F21" s="51">
+        <f>IF((F22+$C$8)&gt;0,$C$8*F14/(F22+$C$8),"n/a")</f>
+        <v/>
+      </c>
+      <c r="G21" s="51">
+        <f>IF((G22+$C$8)&gt;0,$C$8*G14/(G22+$C$8),"n/a")</f>
+        <v/>
+      </c>
+      <c r="H21" s="51">
+        <f>IF((H22+$C$8)&gt;0,$C$8*H14/(H22+$C$8),"n/a")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="C22" s="52">
+        <f>C28-C16*C18-$C$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="52">
+        <f>D28-D16*D18-$C$8</f>
+        <v/>
+      </c>
+      <c r="E22" s="52">
+        <f>E28-E16*E18-$C$8</f>
+        <v/>
+      </c>
+      <c r="F22" s="52">
+        <f>F28-F16*F18-$C$8</f>
+        <v/>
+      </c>
+      <c r="G22" s="52">
+        <f>G28-G16*G18-$C$8</f>
+        <v/>
+      </c>
+      <c r="H22" s="52">
+        <f>H28-H16*H18-$C$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>EBITDA %</t>
         </is>
       </c>
-      <c r="C19" s="51">
-        <f>((((C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-C7*C5*Channels!$P$9)-C6*C5*Channels!$R$9-C9*C6*C5*Channels!$S$9-C5*Channels!$T$9-C5*Channels!$U$9)-'P&amp;L'!$C$8*(C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))-'P&amp;L'!$C$13)/(C6*C5*(Channels!$L$9-C8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="D19" s="51">
-        <f>((((D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-D7*D5*Channels!$P$9)-D6*D5*Channels!$R$9-D9*D6*D5*Channels!$S$9-D5*Channels!$T$9-D5*Channels!$U$9)-'P&amp;L'!$C$8*(D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))-'P&amp;L'!$C$13)/(D6*D5*(Channels!$L$9-D8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
-      </c>
-      <c r="E19" s="51">
-        <f>((((E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-E7*E5*Channels!$P$9)-E6*E5*Channels!$R$9-E9*E6*E5*Channels!$S$9-E5*Channels!$T$9-E5*Channels!$U$9)-'P&amp;L'!$C$8*(E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))-'P&amp;L'!$C$13)/(E6*E5*(Channels!$L$9-E8*Channels!$M$9-Channels!$N$9))</f>
-        <v/>
+      <c r="C23" s="53">
+        <f>C22/C18</f>
+        <v/>
+      </c>
+      <c r="D23" s="53">
+        <f>D22/D18</f>
+        <v/>
+      </c>
+      <c r="E23" s="53">
+        <f>E22/E18</f>
+        <v/>
+      </c>
+      <c r="F23" s="53">
+        <f>F22/F18</f>
+        <v/>
+      </c>
+      <c r="G23" s="53">
+        <f>G22/G18</f>
+        <v/>
+      </c>
+      <c r="H23" s="53">
+        <f>H22/H18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" hidden="1">
+      <c r="C25">
+        <f>C12/$C$5</f>
+        <v/>
+      </c>
+      <c r="D25">
+        <f>D12/$C$5</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>E12/$C$5</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>F12/$C$5</f>
+        <v/>
+      </c>
+      <c r="G25">
+        <f>G12/$C$5</f>
+        <v/>
+      </c>
+      <c r="H25">
+        <f>H12/$C$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" hidden="1">
+      <c r="C26">
+        <f>C13/$C$6</f>
+        <v/>
+      </c>
+      <c r="D26">
+        <f>D13/$C$6</f>
+        <v/>
+      </c>
+      <c r="E26">
+        <f>E13/$C$6</f>
+        <v/>
+      </c>
+      <c r="F26">
+        <f>F13/$C$6</f>
+        <v/>
+      </c>
+      <c r="G26">
+        <f>G13/$C$6</f>
+        <v/>
+      </c>
+      <c r="H26">
+        <f>H13/$C$6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" hidden="1">
+      <c r="C27">
+        <f>C14/$C$7</f>
+        <v/>
+      </c>
+      <c r="D27">
+        <f>D14/$C$7</f>
+        <v/>
+      </c>
+      <c r="E27">
+        <f>E14/$C$7</f>
+        <v/>
+      </c>
+      <c r="F27">
+        <f>F14/$C$7</f>
+        <v/>
+      </c>
+      <c r="G27">
+        <f>G14/$C$7</f>
+        <v/>
+      </c>
+      <c r="H27">
+        <f>H14/$C$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" hidden="1">
+      <c r="C28">
+        <f>(C18-C26*C27*Channels!$P$9)-C25*C27*Channels!$R$9-C25*C27*Channels!$S$9-C27*Channels!$T$9-C27*Channels!$U$9</f>
+        <v/>
+      </c>
+      <c r="D28">
+        <f>(D18-D26*D27*Channels!$P$9)-D25*D27*Channels!$R$9-D25*D27*Channels!$S$9-D27*Channels!$T$9-D27*Channels!$U$9</f>
+        <v/>
+      </c>
+      <c r="E28">
+        <f>(E18-E26*E27*Channels!$P$9)-E25*E27*Channels!$R$9-E25*E27*Channels!$S$9-E27*Channels!$T$9-E27*Channels!$U$9</f>
+        <v/>
+      </c>
+      <c r="F28">
+        <f>(F18-F26*F27*Channels!$P$9)-F25*F27*Channels!$R$9-F25*F27*Channels!$S$9-F27*Channels!$T$9-F27*Channels!$U$9</f>
+        <v/>
+      </c>
+      <c r="G28">
+        <f>(G18-G26*G27*Channels!$P$9)-G25*G27*Channels!$R$9-G25*G27*Channels!$S$9-G27*Channels!$T$9-G27*Channels!$U$9</f>
+        <v/>
+      </c>
+      <c r="H28">
+        <f>(H18-H26*H27*Channels!$P$9)-H25*H27*Channels!$R$9-H25*H27*Channels!$S$9-H27*Channels!$T$9-H27*Channels!$U$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="54" t="inlineStr">
+        <is>
+          <t>Edit any yellow dial and the whole column recomputes. To add a scenario, copy column H and edit its dials.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C18">
-    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+  <conditionalFormatting sqref="C18:H18">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>C18=MAX($C18:$H18)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19:H19">
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>C19=MAX($C19:$H19)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C20:H20">
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>C20=MAX($C20:$H20)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C22:H22">
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>C22=MAX($C22:$H22)</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="1">
+    <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D18">
-    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
+  <conditionalFormatting sqref="C23:H23">
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>C23=MAX($C23:$H23)</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="1">
+    <cfRule type="cellIs" priority="10" operator="greaterThanOrEqual" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
-    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="1">
-      <formula>0</formula>
+  <conditionalFormatting sqref="C21:H21">
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>C21=MIN($C21:$H21)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3016,169 +3427,169 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="52" t="inlineStr"/>
+      <c r="B4" s="55" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B5" s="56" t="inlineStr">
         <is>
           <t>The waterfall</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B6" s="57" t="inlineStr">
         <is>
           <t>Gross Sales − Trade − Returns = NET SALES</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="54" t="inlineStr">
+      <c r="B7" s="57" t="inlineStr">
         <is>
           <t>Net Sales − COGS = GROSS PROFIT   (Gross Margin %)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="54" t="inlineStr">
+      <c r="B8" s="57" t="inlineStr">
         <is>
           <t>Gross Profit − fulfillment − fees − channel ad − slotting = CONTRIBUTION MARGIN  (CM %)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="54" t="inlineStr">
+      <c r="B9" s="57" t="inlineStr">
         <is>
           <t>Contribution − brand marketing − sales − G&amp;A − R&amp;D = EBITDA   (EBITDA %)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="52" t="inlineStr"/>
+      <c r="B10" s="55" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" s="53" t="inlineStr">
+      <c r="B11" s="56" t="inlineStr">
         <is>
           <t>Why contribution margin is the number to watch</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="52" t="inlineStr">
+      <c r="B12" s="55" t="inlineStr">
         <is>
           <t>Gross margin flatters DTC and Amazon because their shelf prices are high — but those channels</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="52" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
         <is>
           <t>bleed it back through referral fees, fulfillment and customer acquisition. Contribution margin is</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="52" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
         <is>
           <t>what each channel actually leaves to cover corporate overhead. Manage the mix on contribution.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="52" t="inlineStr"/>
+      <c r="B15" s="55" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="53" t="inlineStr">
+      <c r="B16" s="56" t="inlineStr">
         <is>
           <t>Where the levers are (see the Sensitivity &amp; tornado)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="52" t="inlineStr">
+      <c r="B17" s="55" t="inlineStr">
         <is>
           <t>• COGS — every cent off a can flows straight to EBITDA at full volume.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="52" t="inlineStr">
+      <c r="B18" s="55" t="inlineStr">
         <is>
           <t>• Price &amp; trade — highest-leverage revenue dials, but trade is sticky once retailers expect it.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="52" t="inlineStr">
+      <c r="B19" s="55" t="inlineStr">
         <is>
           <t>• Mix — shifting volume to higher-contribution channels lifts EBITDA without touching a cost.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="52" t="inlineStr">
+      <c r="B20" s="55" t="inlineStr">
         <is>
           <t>• Volume vs fixed cost — overhead is fixed, so scale is its own lever (see break-even).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="52" t="inlineStr"/>
+      <c r="B21" s="55" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="B22" s="53" t="inlineStr">
+      <c r="B22" s="56" t="inlineStr">
         <is>
           <t>Sheet map</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="52" t="inlineStr">
+      <c r="B23" s="55" t="inlineStr">
         <is>
           <t>P&amp;L          – assumptions (yellow) + the blended statement, per-case and % of net sales.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="52" t="inlineStr">
+      <c r="B24" s="55" t="inlineStr">
         <is>
           <t>COGS_BOM     – bill of materials → landed cost per can; feeds every channel.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="52" t="inlineStr">
+      <c r="B25" s="55" t="inlineStr">
         <is>
           <t>Channels     – the revenue engine; one column block per route to market, totals feed the P&amp;L.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="52" t="inlineStr">
+      <c r="B26" s="55" t="inlineStr">
         <is>
           <t>Sensitivity  – EBITDA % across a price × COGS grid, coloured as a heatmap.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="52" t="inlineStr">
-        <is>
-          <t>Scenarios    – Base / Bull / Bear via editable multipliers on the channel totals.</t>
+      <c r="B27" s="55" t="inlineStr">
+        <is>
+          <t>Scenario Lab – compare many full plans side by side; edit each column's dials, best in row turns green.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="52" t="inlineStr"/>
+      <c r="B28" s="55" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="B29" s="55" t="inlineStr">
+      <c r="B29" s="58" t="inlineStr">
         <is>
           <t>Defaults model Organika MÜV Sparkling Electrolytes (355 ml can, zero-sugar; magnesium bisglycinate</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="55" t="inlineStr">
+      <c r="B30" s="58" t="inlineStr">
         <is>
           <t>+ Fibersol prebiotic fiber) as a representative premium functional beverage. Replace with your actuals.</t>
         </is>

</xml_diff>